<commit_message>
v2 import hardening: warehouse-ensure, dedup, wipe, parallel-safe tests
Fixes found before the prod cutover:
- get_service/get_unit now ensure a warehouse on the FOUND branch too
  (pre-existing v1 services were warehouse-less → empty-«Де» rows lost)
- nomenclature + persons caches seed from DB → re-import reuses instead
  of creating duplicates (real prod re-import bug)
- POST /api/admin/v2/wipe — clears v2 inventory (assignments, movements,
  instances, nomenclature) for iterative re-import
- Tests: disjoint fixture names + delta assertions (parallel-safe);
  destructive wipe/idempotency test gated behind RUN_WIPE_TEST

Full suite stable 3× (89 Playwright, 44 pytest).

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tests/e2e/tests/fixtures/import_v2_items.xlsx
+++ b/tests/e2e/tests/fixtures/import_v2_items.xlsx
@@ -461,12 +461,12 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Бушлат</t>
+          <t>БушлатA</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Речова</t>
+          <t>ImpSvcA</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -487,7 +487,7 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>1 рота Петренко</t>
+          <t>ImpUnitA Петренко</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
@@ -499,17 +499,17 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>АК-74</t>
+          <t>АК-A</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>РАО</t>
+          <t>ImpSvcA</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>AK-IMP-1</t>
+          <t>AK-IMP-A</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -525,19 +525,19 @@
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>1 рота</t>
+          <t>ImpUnitA</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Патрони 5.45</t>
+          <t>ПатрониA</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>РАО</t>
+          <t>ImpRaoA</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">

</xml_diff>